<commit_message>
docs(fix): fichier non sauvegardé, écart entre les fichiers
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-09-product-backlog-v2.xlsx
+++ b/docs/cadrage/equipe-09-product-backlog-v2.xlsx
@@ -314,9 +314,6 @@
 T: chaque réponse comparée, statut bon/mauvais enregistré</t>
   </si>
   <si>
-    <t xml:space="preserve">S3</t>
-  </si>
-  <si>
     <t xml:space="preserve">Todo</t>
   </si>
   <si>
@@ -331,6 +328,9 @@
 T: score /10 affiché + 10 questions avec corrections détaillées</t>
   </si>
   <si>
+    <t xml:space="preserve">S3</t>
+  </si>
+  <si>
     <t xml:space="preserve">US-06</t>
   </si>
   <si>
@@ -342,45 +342,45 @@
 T: liste des quizz triés par date desc, avec titre/date/score/refaire</t>
   </si>
   <si>
+    <t xml:space="preserve">US-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En tant qu'étudiant·e, je veux réinitialiser mon mot de passe via email, afin de pouvoir récupérer mon compte sans support.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SHOULD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[1 critère type : lien magique valide 24 h, redirect /reset-password]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backlog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En tant qu'étudiant·e, je veux une bibliothèque pour mes cours uploadés, afin de retrouver vite mes PDF d'un semestre.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[1 critère type : page /library liste cours avec date, titre, nb quizz]</t>
+  </si>
+  <si>
     <t xml:space="preserve">S4</t>
   </si>
   <si>
-    <t xml:space="preserve">US-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En tant qu'étudiant·e, je veux réinitialiser mon mot de passe via email, afin de pouvoir récupérer mon compte sans support.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SHOULD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[1 critère type : lien magique valide 24 h, redirect /reset-password]</t>
+    <t xml:space="preserve">US-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En tant qu'étudiant·e, je veux choisir le niveau de difficulté et le nombre de questions (5-20), afin d'adapter à mon temps disponible.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[1 critère type : 3 niveaux (facile/moyen/dur) + slider 5-20 sur /quiz]</t>
   </si>
   <si>
     <t xml:space="preserve">S6</t>
   </si>
   <si>
-    <t xml:space="preserve">Backlog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En tant qu'étudiant·e, je veux une bibliothèque pour mes cours uploadés, afin de retrouver vite mes PDF d'un semestre.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[1 critère type : page /library liste cours avec date, titre, nb quizz]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En tant qu'étudiant·e, je veux choisir le niveau de difficulté et le nombre de questions (5-20), afin d'adapter à mon temps disponible.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[1 critère type : 3 niveaux (facile/moyen/dur) + slider 5-20 sur /quiz]</t>
-  </si>
-  <si>
     <t xml:space="preserve">US-10</t>
   </si>
   <si>
@@ -390,16 +390,16 @@
     <t xml:space="preserve">[1 critère type : toggle ON/OFF + slider 10-30 s configurable]</t>
   </si>
   <si>
+    <t xml:space="preserve">US-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En tant qu'étudiant·e, je veux un dashboard de progression par chapitre, afin de cibler mes révisions sur mes lacunes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[1 critère type : page /dashboard avec graphique en barres score / chap.]</t>
+  </si>
+  <si>
     <t xml:space="preserve">S7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En tant qu'étudiant·e, je veux un dashboard de progression par chapitre, afin de cibler mes révisions sur mes lacunes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[1 critère type : page /dashboard avec graphique en barres score / chap.]</t>
   </si>
   <si>
     <t xml:space="preserve">US-12</t>
@@ -1066,164 +1066,168 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="25" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="28" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="28" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="29" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="30" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="30" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1482,42 +1486,42 @@
   <dimension ref="B2:B21"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="90"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="90"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="85.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="29.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="7" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="8" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1540,76 +1544,76 @@
   <dimension ref="B2:C13"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="68.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="68.57"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="10" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="12" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="13" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="13" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="14" t="n">
         <v>46203.375</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="13" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="15" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="8" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1632,164 +1636,164 @@
   <dimension ref="A1:E13"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="16" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="E6" s="17" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="19" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="19" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="19" t="n">
         <v>47</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="19" t="n">
         <v>22</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E11" s="19" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="D12" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E12" s="19" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="C13" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="D13" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="E13" s="19" t="n">
         <v>18</v>
       </c>
     </row>
@@ -1812,953 +1816,953 @@
   <dimension ref="A1:K35"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="16" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="10" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="10" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="10" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="F9" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="G9" s="16" t="s">
+      <c r="G9" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="I9" s="16" t="s">
+      <c r="I9" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="J9" s="16" t="s">
+      <c r="J9" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="K9" s="16" t="s">
+      <c r="K9" s="17" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
+      <c r="A10" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C10" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="F10" s="24" t="n">
+      <c r="F10" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="G10" s="24" t="s">
+      <c r="G10" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="H10" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I10" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J10" s="24" t="s">
+      <c r="H10" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I10" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J10" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="K10" s="24" t="s">
+      <c r="K10" s="25" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="s">
+      <c r="A11" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="C11" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="D11" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="E11" s="25" t="s">
+      <c r="E11" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="24" t="n">
+      <c r="F11" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="24" t="s">
+      <c r="G11" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="H11" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I11" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J11" s="24" t="s">
+      <c r="H11" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I11" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J11" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="K11" s="24" t="s">
+      <c r="K11" s="25" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23" t="s">
+      <c r="A12" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="24" t="s">
+      <c r="C12" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="D12" s="24" t="s">
+      <c r="D12" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="E12" s="25" t="s">
+      <c r="E12" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="F12" s="24" t="n">
+      <c r="F12" s="25" t="n">
         <v>8</v>
       </c>
-      <c r="G12" s="24" t="s">
+      <c r="G12" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="H12" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I12" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J12" s="24" t="s">
+      <c r="H12" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I12" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J12" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="K12" s="24" t="s">
+      <c r="K12" s="25" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="23" t="s">
+      <c r="A13" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="24" t="s">
+      <c r="C13" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="E13" s="25" t="s">
+      <c r="E13" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="F13" s="24" t="n">
+      <c r="F13" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="G13" s="24" t="s">
+      <c r="G13" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="H13" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I13" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J13" s="24" t="s">
+      <c r="H13" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I13" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J13" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="K13" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="24" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="24" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="23" t="s">
+      <c r="B14" s="25" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="B14" s="24" t="s">
+      <c r="D14" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="F14" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="H14" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I14" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J14" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="K14" s="25" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="E15" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="F15" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="25" t="s">
+        <v>100</v>
+      </c>
+      <c r="H15" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I15" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J15" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="K15" s="25" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="B16" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="D16" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="E16" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="F16" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="H16" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I16" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J16" s="25" t="s">
+        <v>97</v>
+      </c>
+      <c r="K16" s="25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="B17" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="E17" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="F17" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="G17" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="H17" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I17" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J17" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="K17" s="25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="G18" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="H18" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I18" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J18" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="K18" s="25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="B19" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="24" t="s">
-        <v>96</v>
-      </c>
-      <c r="D14" s="24" t="s">
+      <c r="C19" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="D19" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="E14" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="F14" s="24" t="n">
+      <c r="E19" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="F19" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="24" t="s">
-        <v>97</v>
-      </c>
-      <c r="H14" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I14" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J14" s="24" t="s">
-        <v>93</v>
-      </c>
-      <c r="K14" s="24" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23" t="s">
-        <v>98</v>
-      </c>
-      <c r="B15" s="24" t="s">
+      <c r="G19" s="25" t="s">
+        <v>116</v>
+      </c>
+      <c r="H19" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I19" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J19" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="K19" s="25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="24" t="s">
+        <v>117</v>
+      </c>
+      <c r="B20" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="24" t="s">
-        <v>99</v>
-      </c>
-      <c r="D15" s="24" t="s">
+      <c r="C20" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="D20" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="E15" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="F15" s="24" t="n">
+      <c r="E20" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="F20" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="G20" s="25" t="s">
+        <v>119</v>
+      </c>
+      <c r="H20" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I20" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J20" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="K20" s="25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="B21" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="D21" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="E21" s="27" t="s">
+        <v>103</v>
+      </c>
+      <c r="F21" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="H21" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="I21" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="J21" s="25" t="s">
+        <v>125</v>
+      </c>
+      <c r="K21" s="25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="87" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="B22" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" s="28" t="s">
+        <v>127</v>
+      </c>
+      <c r="D22" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="E22" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="F22" s="25" t="n">
+        <v>7</v>
+      </c>
+      <c r="G22" s="28" t="s">
+        <v>129</v>
+      </c>
+      <c r="H22" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="I22" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="J22" s="28" t="s">
+        <v>120</v>
+      </c>
+      <c r="K22" s="28" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="29" t="s">
+        <v>130</v>
+      </c>
+      <c r="B23" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="25" t="s">
+        <v>131</v>
+      </c>
+      <c r="D23" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="E23" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="F23" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="24" t="s">
-        <v>100</v>
-      </c>
-      <c r="H15" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I15" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J15" s="24" t="s">
-        <v>101</v>
-      </c>
-      <c r="K15" s="24" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="s">
-        <v>102</v>
-      </c>
-      <c r="B16" s="24" t="s">
+      <c r="G23" s="28" t="s">
+        <v>132</v>
+      </c>
+      <c r="H23" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="I23" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="J23" s="28" t="s">
+        <v>120</v>
+      </c>
+      <c r="K23" s="28" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="24" t="s">
+        <v>133</v>
+      </c>
+      <c r="B24" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="24" t="s">
-        <v>103</v>
-      </c>
-      <c r="D16" s="24" t="s">
+      <c r="C24" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="D24" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="E16" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="F16" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="G16" s="24" t="s">
+      <c r="E24" s="31" t="s">
+        <v>135</v>
+      </c>
+      <c r="F24" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="G24" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="H24" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I24" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J24" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="K24" s="25" t="s">
         <v>105</v>
       </c>
-      <c r="H16" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I16" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J16" s="24" t="s">
-        <v>106</v>
-      </c>
-      <c r="K16" s="24" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="23" t="s">
-        <v>108</v>
-      </c>
-      <c r="B17" s="24" t="s">
+    </row>
+    <row r="25" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="B25" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="24" t="s">
-        <v>109</v>
-      </c>
-      <c r="D17" s="24" t="s">
+      <c r="C25" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="D25" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="E17" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="F17" s="24" t="n">
+      <c r="E25" s="31" t="s">
+        <v>135</v>
+      </c>
+      <c r="F25" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="G25" s="25" t="s">
+        <v>140</v>
+      </c>
+      <c r="H25" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I25" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J25" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="K25" s="25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="24" t="s">
+        <v>141</v>
+      </c>
+      <c r="B26" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="25" t="s">
+        <v>142</v>
+      </c>
+      <c r="D26" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="E26" s="31" t="s">
+        <v>135</v>
+      </c>
+      <c r="F26" s="25" t="n">
+        <v>13</v>
+      </c>
+      <c r="G26" s="25" t="s">
+        <v>144</v>
+      </c>
+      <c r="H26" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I26" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J26" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="K26" s="25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="24" t="s">
+        <v>145</v>
+      </c>
+      <c r="B27" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="D27" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="E27" s="31" t="s">
+        <v>135</v>
+      </c>
+      <c r="F27" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="G27" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="H27" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I27" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J27" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="K27" s="25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="24" t="s">
+        <v>148</v>
+      </c>
+      <c r="B28" s="25" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" s="25" t="s">
+        <v>149</v>
+      </c>
+      <c r="D28" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="E28" s="31" t="s">
+        <v>135</v>
+      </c>
+      <c r="F28" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="G17" s="24" t="s">
-        <v>110</v>
-      </c>
-      <c r="H17" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I17" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J17" s="24" t="s">
-        <v>106</v>
-      </c>
-      <c r="K17" s="24" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="23" t="s">
-        <v>111</v>
-      </c>
-      <c r="B18" s="24" t="s">
+      <c r="G28" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="H28" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="I28" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J28" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="K28" s="25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="29" t="s">
+        <v>151</v>
+      </c>
+      <c r="B29" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" s="28" t="s">
+        <v>152</v>
+      </c>
+      <c r="D29" s="28" t="s">
+        <v>128</v>
+      </c>
+      <c r="E29" s="32" t="s">
+        <v>135</v>
+      </c>
+      <c r="F29" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="G29" s="28" t="s">
+        <v>153</v>
+      </c>
+      <c r="H29" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="I29" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="J29" s="28" t="s">
+        <v>137</v>
+      </c>
+      <c r="K29" s="28" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="24" t="s">
+        <v>154</v>
+      </c>
+      <c r="B30" s="25" t="s">
+        <v>30</v>
+      </c>
+      <c r="C30" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="D30" s="25" t="s">
+        <v>156</v>
+      </c>
+      <c r="E30" s="33" t="s">
+        <v>157</v>
+      </c>
+      <c r="F30" s="25" t="n">
+        <v>13</v>
+      </c>
+      <c r="G30" s="25" t="s">
+        <v>158</v>
+      </c>
+      <c r="H30" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I30" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J30" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="K30" s="25" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="B31" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="24" t="s">
-        <v>112</v>
-      </c>
-      <c r="D18" s="24" t="s">
+      <c r="C31" s="25" t="s">
+        <v>161</v>
+      </c>
+      <c r="D31" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="E18" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="F18" s="24" t="n">
-        <v>5</v>
-      </c>
-      <c r="G18" s="24" t="s">
-        <v>113</v>
-      </c>
-      <c r="H18" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I18" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J18" s="24" t="s">
-        <v>106</v>
-      </c>
-      <c r="K18" s="24" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="B19" s="24" t="s">
+      <c r="E31" s="33" t="s">
+        <v>157</v>
+      </c>
+      <c r="F31" s="25" t="n">
+        <v>21</v>
+      </c>
+      <c r="G31" s="25" t="s">
+        <v>162</v>
+      </c>
+      <c r="H31" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I31" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J31" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="K31" s="25" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="24" t="s">
+        <v>163</v>
+      </c>
+      <c r="B32" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="24" t="s">
-        <v>115</v>
-      </c>
-      <c r="D19" s="24" t="s">
+      <c r="C32" s="25" t="s">
+        <v>164</v>
+      </c>
+      <c r="D32" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="E19" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="F19" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="G19" s="24" t="s">
-        <v>116</v>
-      </c>
-      <c r="H19" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I19" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J19" s="24" t="s">
-        <v>117</v>
-      </c>
-      <c r="K19" s="24" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="B20" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="C20" s="24" t="s">
-        <v>119</v>
-      </c>
-      <c r="D20" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="E20" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="F20" s="24" t="n">
-        <v>5</v>
-      </c>
-      <c r="G20" s="24" t="s">
-        <v>120</v>
-      </c>
-      <c r="H20" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I20" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J20" s="24" t="s">
-        <v>117</v>
-      </c>
-      <c r="K20" s="24" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="B21" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="C21" s="24" t="s">
-        <v>122</v>
-      </c>
-      <c r="D21" s="24" t="s">
-        <v>123</v>
-      </c>
-      <c r="E21" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="F21" s="24" t="n">
-        <v>5</v>
-      </c>
-      <c r="G21" s="24" t="s">
-        <v>124</v>
-      </c>
-      <c r="H21" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="I21" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="J21" s="24" t="s">
-        <v>125</v>
-      </c>
-      <c r="K21" s="24" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="87" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="28" t="s">
-        <v>126</v>
-      </c>
-      <c r="B22" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="C22" s="27" t="s">
+      <c r="E32" s="33" t="s">
+        <v>157</v>
+      </c>
+      <c r="F32" s="25" t="n">
+        <v>13</v>
+      </c>
+      <c r="G32" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="H32" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I32" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J32" s="25" t="s">
+        <v>137</v>
+      </c>
+      <c r="K32" s="25" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="69.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="29"/>
+      <c r="B33" s="25"/>
+      <c r="C33" s="28" t="s">
         <v>127</v>
       </c>
-      <c r="D22" s="27" t="s">
+      <c r="D33" s="28" t="s">
         <v>128</v>
       </c>
-      <c r="E22" s="29" t="s">
-        <v>104</v>
-      </c>
-      <c r="F22" s="24" t="n">
-        <v>7</v>
-      </c>
-      <c r="G22" s="27" t="s">
-        <v>129</v>
-      </c>
-      <c r="H22" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="I22" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="J22" s="27" t="s">
-        <v>117</v>
-      </c>
-      <c r="K22" s="27" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="28" t="s">
+      <c r="E33" s="33"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="25"/>
+      <c r="I33" s="25"/>
+      <c r="J33" s="25"/>
+      <c r="K33" s="25"/>
+    </row>
+    <row r="34" customFormat="false" ht="69.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="29" t="s">
         <v>130</v>
       </c>
-      <c r="B23" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="C23" s="24" t="s">
+      <c r="B34" s="25"/>
+      <c r="C34" s="28" t="s">
         <v>131</v>
       </c>
-      <c r="D23" s="27" t="s">
+      <c r="D34" s="28" t="s">
         <v>128</v>
       </c>
-      <c r="E23" s="29" t="s">
-        <v>104</v>
-      </c>
-      <c r="F23" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="G23" s="27" t="s">
-        <v>132</v>
-      </c>
-      <c r="H23" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="I23" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="J23" s="27" t="s">
-        <v>117</v>
-      </c>
-      <c r="K23" s="27" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="23" t="s">
-        <v>133</v>
-      </c>
-      <c r="B24" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="C24" s="24" t="s">
-        <v>134</v>
-      </c>
-      <c r="D24" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="E24" s="30" t="s">
-        <v>135</v>
-      </c>
-      <c r="F24" s="24" t="n">
-        <v>5</v>
-      </c>
-      <c r="G24" s="24" t="s">
-        <v>136</v>
-      </c>
-      <c r="H24" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I24" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J24" s="24" t="s">
+      <c r="E34" s="33"/>
+      <c r="F34" s="25"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="25"/>
+      <c r="I34" s="25"/>
+      <c r="J34" s="25"/>
+      <c r="K34" s="25"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="34" t="s">
+        <v>166</v>
+      </c>
+      <c r="B35" s="35"/>
+      <c r="C35" s="35"/>
+      <c r="D35" s="35"/>
+      <c r="E35" s="35"/>
+      <c r="F35" s="34" t="n">
         <v>137</v>
       </c>
-      <c r="K24" s="24" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="23" t="s">
-        <v>138</v>
-      </c>
-      <c r="B25" s="24" t="s">
-        <v>34</v>
-      </c>
-      <c r="C25" s="24" t="s">
-        <v>139</v>
-      </c>
-      <c r="D25" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="E25" s="30" t="s">
-        <v>135</v>
-      </c>
-      <c r="F25" s="24" t="n">
-        <v>8</v>
-      </c>
-      <c r="G25" s="24" t="s">
-        <v>140</v>
-      </c>
-      <c r="H25" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I25" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J25" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="K25" s="24" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="B26" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="C26" s="24" t="s">
-        <v>142</v>
-      </c>
-      <c r="D26" s="24" t="s">
-        <v>143</v>
-      </c>
-      <c r="E26" s="30" t="s">
-        <v>135</v>
-      </c>
-      <c r="F26" s="24" t="n">
-        <v>13</v>
-      </c>
-      <c r="G26" s="24" t="s">
-        <v>144</v>
-      </c>
-      <c r="H26" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I26" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J26" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="K26" s="24" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="B27" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="C27" s="24" t="s">
-        <v>146</v>
-      </c>
-      <c r="D27" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="E27" s="30" t="s">
-        <v>135</v>
-      </c>
-      <c r="F27" s="24" t="n">
-        <v>8</v>
-      </c>
-      <c r="G27" s="24" t="s">
-        <v>147</v>
-      </c>
-      <c r="H27" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I27" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J27" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="K27" s="24" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="B28" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="C28" s="24" t="s">
-        <v>149</v>
-      </c>
-      <c r="D28" s="24" t="s">
-        <v>123</v>
-      </c>
-      <c r="E28" s="30" t="s">
-        <v>135</v>
-      </c>
-      <c r="F28" s="24" t="n">
-        <v>5</v>
-      </c>
-      <c r="G28" s="27" t="s">
-        <v>150</v>
-      </c>
-      <c r="H28" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="I28" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J28" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="K28" s="24" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="28" t="s">
-        <v>151</v>
-      </c>
-      <c r="B29" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="C29" s="27" t="s">
-        <v>152</v>
-      </c>
-      <c r="D29" s="27" t="s">
-        <v>128</v>
-      </c>
-      <c r="E29" s="31" t="s">
-        <v>135</v>
-      </c>
-      <c r="F29" s="24" t="n">
-        <v>8</v>
-      </c>
-      <c r="G29" s="27" t="s">
-        <v>153</v>
-      </c>
-      <c r="H29" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="I29" s="27" t="s">
-        <v>80</v>
-      </c>
-      <c r="J29" s="27" t="s">
-        <v>137</v>
-      </c>
-      <c r="K29" s="27" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="23" t="s">
-        <v>154</v>
-      </c>
-      <c r="B30" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="C30" s="24" t="s">
-        <v>155</v>
-      </c>
-      <c r="D30" s="24" t="s">
-        <v>156</v>
-      </c>
-      <c r="E30" s="32" t="s">
-        <v>157</v>
-      </c>
-      <c r="F30" s="24" t="n">
-        <v>13</v>
-      </c>
-      <c r="G30" s="24" t="s">
-        <v>158</v>
-      </c>
-      <c r="H30" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I30" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J30" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="K30" s="24" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="23" t="s">
-        <v>160</v>
-      </c>
-      <c r="B31" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="C31" s="24" t="s">
-        <v>161</v>
-      </c>
-      <c r="D31" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="E31" s="32" t="s">
-        <v>157</v>
-      </c>
-      <c r="F31" s="24" t="n">
-        <v>21</v>
-      </c>
-      <c r="G31" s="24" t="s">
-        <v>162</v>
-      </c>
-      <c r="H31" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I31" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J31" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="K31" s="24" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="23" t="s">
-        <v>163</v>
-      </c>
-      <c r="B32" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="C32" s="24" t="s">
-        <v>164</v>
-      </c>
-      <c r="D32" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="E32" s="32" t="s">
-        <v>157</v>
-      </c>
-      <c r="F32" s="24" t="n">
-        <v>13</v>
-      </c>
-      <c r="G32" s="24" t="s">
-        <v>165</v>
-      </c>
-      <c r="H32" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="I32" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="J32" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="K32" s="24" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="69.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="28"/>
-      <c r="B33" s="24"/>
-      <c r="C33" s="27" t="s">
-        <v>127</v>
-      </c>
-      <c r="D33" s="27" t="s">
-        <v>128</v>
-      </c>
-      <c r="E33" s="32"/>
-      <c r="F33" s="24"/>
-      <c r="G33" s="24"/>
-      <c r="H33" s="24"/>
-      <c r="I33" s="24"/>
-      <c r="J33" s="24"/>
-      <c r="K33" s="24"/>
-    </row>
-    <row r="34" customFormat="false" ht="69.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="28" t="s">
-        <v>130</v>
-      </c>
-      <c r="B34" s="24"/>
-      <c r="C34" s="27" t="s">
-        <v>131</v>
-      </c>
-      <c r="D34" s="27" t="s">
-        <v>128</v>
-      </c>
-      <c r="E34" s="32"/>
-      <c r="F34" s="24"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="24"/>
-      <c r="I34" s="24"/>
-      <c r="J34" s="24"/>
-      <c r="K34" s="24"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="33" t="s">
-        <v>166</v>
-      </c>
-      <c r="B35" s="34"/>
-      <c r="C35" s="34"/>
-      <c r="D35" s="34"/>
-      <c r="E35" s="34"/>
-      <c r="F35" s="33" t="n">
-        <v>137</v>
-      </c>
-      <c r="G35" s="35" t="s">
+      <c r="G35" s="36" t="s">
         <v>167</v>
       </c>
-      <c r="H35" s="34"/>
-      <c r="I35" s="34"/>
-      <c r="J35" s="34"/>
-      <c r="K35" s="34"/>
+      <c r="H35" s="35"/>
+      <c r="I35" s="35"/>
+      <c r="J35" s="35"/>
+      <c r="K35" s="35"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2779,121 +2783,121 @@
   <dimension ref="A1:A28"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="95"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="16" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="37" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="10" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="37" t="s">
+      <c r="A7" s="38" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="37" t="s">
+      <c r="A8" s="38" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="37" t="s">
+      <c r="A9" s="38" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="37" t="s">
+      <c r="A10" s="38" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="37" t="s">
+      <c r="A11" s="38" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="37" t="s">
+      <c r="A12" s="38" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="37" t="s">
+      <c r="A13" s="38" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="37" t="s">
+      <c r="A14" s="38" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="37" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="10" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="37" t="s">
+      <c r="A20" s="38" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="37" t="s">
+      <c r="A21" s="38" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="37" t="s">
+      <c r="A22" s="38" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="37" t="s">
+      <c r="A23" s="38" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="37" t="s">
+      <c r="A24" s="38" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="37" t="s">
+      <c r="A25" s="38" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="37" t="s">
+      <c r="A26" s="38" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="37" t="s">
+      <c r="A27" s="38" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="37" t="s">
+      <c r="A28" s="38" t="s">
         <v>190</v>
       </c>
     </row>
@@ -2916,141 +2920,141 @@
   <dimension ref="A2:D15"/>
   <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="40"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="10" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16"/>
-      <c r="B5" s="16" t="s">
+      <c r="A5" s="17"/>
+      <c r="B5" s="17" t="s">
         <v>193</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="17" t="s">
         <v>194</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="39" t="s">
         <v>196</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="D6" s="38" t="s">
+      <c r="D6" s="39" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="39" t="s">
         <v>199</v>
       </c>
-      <c r="C7" s="39" t="s">
+      <c r="C7" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="D7" s="38" t="s">
+      <c r="D7" s="39" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="48.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="39" t="s">
         <v>200</v>
       </c>
-      <c r="C8" s="39" t="s">
+      <c r="C8" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="D8" s="38" t="s">
+      <c r="D8" s="39" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="39" t="s">
         <v>202</v>
       </c>
-      <c r="C9" s="39" t="s">
+      <c r="C9" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="D9" s="38" t="s">
+      <c r="D9" s="39" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="38" t="s">
+      <c r="B10" s="39" t="s">
         <v>204</v>
       </c>
-      <c r="C10" s="39" t="s">
+      <c r="C10" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="D10" s="38" t="s">
+      <c r="D10" s="39" t="s">
         <v>205</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="44.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="38" t="s">
+      <c r="B11" s="39" t="s">
         <v>206</v>
       </c>
-      <c r="C11" s="39" t="s">
+      <c r="C11" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="D11" s="38" t="s">
+      <c r="D11" s="39" t="s">
         <v>207</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="38" t="s">
+      <c r="B12" s="39" t="s">
         <v>208</v>
       </c>
-      <c r="C12" s="39" t="s">
+      <c r="C12" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="D12" s="38" t="s">
+      <c r="D12" s="39" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="38" t="s">
+      <c r="B13" s="39" t="s">
         <v>210</v>
       </c>
-      <c r="C13" s="39" t="s">
+      <c r="C13" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="D13" s="38" t="s">
+      <c r="D13" s="39" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="38" t="s">
+      <c r="B14" s="39" t="s">
         <v>212</v>
       </c>
-      <c r="C14" s="39" t="s">
+      <c r="C14" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="D14" s="38" t="s">
+      <c r="D14" s="39" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="38" t="s">
+      <c r="B15" s="39" t="s">
         <v>214</v>
       </c>
-      <c r="C15" s="39" t="s">
+      <c r="C15" s="40" t="s">
         <v>197</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="39" t="s">
         <v>215</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(sprint 3): update docs, ajout du sprint3 et données réelles du sprint 2
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-09-product-backlog-v2.xlsx
+++ b/docs/cadrage/equipe-09-product-backlog-v2.xlsx
@@ -314,9 +314,6 @@
 T: chaque réponse comparée, statut bon/mauvais enregistré</t>
   </si>
   <si>
-    <t xml:space="preserve">Todo</t>
-  </si>
-  <si>
     <t xml:space="preserve">US-05</t>
   </si>
   <si>
@@ -331,6 +328,9 @@
     <t xml:space="preserve">S3</t>
   </si>
   <si>
+    <t xml:space="preserve">Todo</t>
+  </si>
+  <si>
     <t xml:space="preserve">US-06</t>
   </si>
   <si>
@@ -354,19 +354,19 @@
     <t xml:space="preserve">[1 critère type : lien magique valide 24 h, redirect /reset-password]</t>
   </si>
   <si>
+    <t xml:space="preserve">US-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En tant qu'étudiant·e, je veux une bibliothèque pour mes cours uploadés, afin de retrouver vite mes PDF d'un semestre.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[1 critère type : page /library liste cours avec date, titre, nb quizz]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S4</t>
+  </si>
+  <si>
     <t xml:space="preserve">Backlog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En tant qu'étudiant·e, je veux une bibliothèque pour mes cours uploadés, afin de retrouver vite mes PDF d'un semestre.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[1 critère type : page /library liste cours avec date, titre, nb quizz]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S4</t>
   </si>
   <si>
     <t xml:space="preserve">US-09</t>
@@ -2041,18 +2041,18 @@
         <v>89</v>
       </c>
       <c r="K13" s="25" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="24" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B14" s="25" t="s">
         <v>42</v>
       </c>
       <c r="C14" s="25" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D14" s="25" t="s">
         <v>77</v>
@@ -2064,19 +2064,19 @@
         <v>3</v>
       </c>
       <c r="G14" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="H14" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I14" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J14" s="25" t="s">
         <v>96</v>
       </c>
-      <c r="H14" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="I14" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="J14" s="25" t="s">
+      <c r="K14" s="25" t="s">
         <v>97</v>
-      </c>
-      <c r="K14" s="25" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2108,10 +2108,10 @@
         <v>80</v>
       </c>
       <c r="J15" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="K15" s="25" t="s">
         <v>97</v>
-      </c>
-      <c r="K15" s="25" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2143,21 +2143,21 @@
         <v>80</v>
       </c>
       <c r="J16" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="K16" s="25" t="s">
         <v>97</v>
-      </c>
-      <c r="K16" s="25" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="24" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B17" s="25" t="s">
         <v>34</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D17" s="25" t="s">
         <v>77</v>
@@ -2169,19 +2169,19 @@
         <v>5</v>
       </c>
       <c r="G17" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="H17" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="I17" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="J17" s="25" t="s">
         <v>108</v>
       </c>
-      <c r="H17" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="I17" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="J17" s="25" t="s">
+      <c r="K17" s="25" t="s">
         <v>109</v>
-      </c>
-      <c r="K17" s="25" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2216,7 +2216,7 @@
         <v>113</v>
       </c>
       <c r="K18" s="25" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2251,7 +2251,7 @@
         <v>113</v>
       </c>
       <c r="K19" s="25" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2286,7 +2286,7 @@
         <v>120</v>
       </c>
       <c r="K20" s="25" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2321,7 +2321,7 @@
         <v>125</v>
       </c>
       <c r="K21" s="25" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="87" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2356,7 +2356,7 @@
         <v>120</v>
       </c>
       <c r="K22" s="28" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2391,7 +2391,7 @@
         <v>120</v>
       </c>
       <c r="K23" s="28" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2426,7 +2426,7 @@
         <v>137</v>
       </c>
       <c r="K24" s="25" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2461,7 +2461,7 @@
         <v>137</v>
       </c>
       <c r="K25" s="25" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2496,7 +2496,7 @@
         <v>137</v>
       </c>
       <c r="K26" s="25" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2531,7 +2531,7 @@
         <v>137</v>
       </c>
       <c r="K27" s="25" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2566,7 +2566,7 @@
         <v>137</v>
       </c>
       <c r="K28" s="25" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2601,7 +2601,7 @@
         <v>137</v>
       </c>
       <c r="K29" s="28" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>